<commit_message>
Adiciona datasets de treino (coletas, desembarque) e atualiza docs/metadados
</commit_message>
<xml_diff>
--- a/data-raw/dados_brutos_eapadados.xlsx
+++ b/data-raw/dados_brutos_eapadados.xlsx
@@ -41,9 +41,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sst_costa_norte" sheetId="33" state="visible" r:id="rId33"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ocorrencias_peixes" sheetId="34" state="visible" r:id="rId34"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cpue_tubarao" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="treino_desembarque" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="treino_coletas" sheetId="37" state="visible" r:id="rId37"/>
   </sheets>
   <externalReferences>
-    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId36"/>
+    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId38"/>
   </externalReferences>
   <definedNames>
     <definedName name="xdata1" hidden="1">22.1714+(ROW(OFFSET(#REF!,0,0,70,1))-1)*0.276907246376812</definedName>
@@ -786,7 +788,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="5.19921875" customWidth="1" min="1" max="1"/>
@@ -1798,6 +1800,60 @@
       <c r="F39" t="inlineStr">
         <is>
           <t>Kruskal-Wallis (CPUE~Year) + serie temporal</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>treino_desembarque</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Desembarque pesqueiro em formato LARGO (2021-2023) - TREINO sintetico</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Porto, Especie, "AAAA - Captura_t", "AAAA - Receita_mil"</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Arrumacao: empilhar/alargar (pivot_longer/wider) -&gt; treino_desembarque</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>treino_coletas</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Coletas com coluna composta (codigo/estacao_periodo) - TREINO sintetico</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>id, codigo_coleta, estacao_periodo, comprimento_cm, peso_g</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Arrumacao: separar (extract/regex) -&gt; treino_coletas</t>
         </is>
       </c>
     </row>
@@ -73504,6 +73560,778 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Porto</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Especie</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>2021 - Captura_t</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>2021 - Receita_mil</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>2022 - Captura_t</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>2022 - Receita_mil</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>2023 - Captura_t</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>2023 - Receita_mil</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Bragança</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Pargo</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>172.6</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2449.3</v>
+      </c>
+      <c r="E2" t="n">
+        <v>184.8</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1843.7</v>
+      </c>
+      <c r="G2" t="n">
+        <v>171.8</v>
+      </c>
+      <c r="H2" t="n">
+        <v>2436.9</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Bragança</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Serra</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>150.2</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1795.4</v>
+      </c>
+      <c r="E3" t="n">
+        <v>145.6</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1533.2</v>
+      </c>
+      <c r="G3" t="n">
+        <v>183.9</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1689.3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Bragança</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Pescada</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>101</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1404.8</v>
+      </c>
+      <c r="E4" t="n">
+        <v>89</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1080.9</v>
+      </c>
+      <c r="G4" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1256.6</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Vigia</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Pargo</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>89.09999999999999</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1014.1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>69.59999999999999</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1092.8</v>
+      </c>
+      <c r="G5" t="n">
+        <v>76.09999999999999</v>
+      </c>
+      <c r="H5" t="n">
+        <v>734.3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Vigia</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Serra</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>61.5</v>
+      </c>
+      <c r="D6" t="n">
+        <v>701.6</v>
+      </c>
+      <c r="E6" t="n">
+        <v>58.8</v>
+      </c>
+      <c r="F6" t="n">
+        <v>547.1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>64.40000000000001</v>
+      </c>
+      <c r="H6" t="n">
+        <v>635.9</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Vigia</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Pescada</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>113.6</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1255.5</v>
+      </c>
+      <c r="E7" t="n">
+        <v>147.3</v>
+      </c>
+      <c r="F7" t="n">
+        <v>2238.7</v>
+      </c>
+      <c r="G7" t="n">
+        <v>130.9</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1354.3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Belém</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Pargo</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>46.8</v>
+      </c>
+      <c r="D8" t="n">
+        <v>495.9</v>
+      </c>
+      <c r="E8" t="n">
+        <v>53</v>
+      </c>
+      <c r="F8" t="n">
+        <v>506.6</v>
+      </c>
+      <c r="G8" t="n">
+        <v>51.6</v>
+      </c>
+      <c r="H8" t="n">
+        <v>500.9</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Belém</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Serra</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>111.4</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1653</v>
+      </c>
+      <c r="E9" t="n">
+        <v>96.90000000000001</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1113.1</v>
+      </c>
+      <c r="G9" t="n">
+        <v>122.3</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1701.5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Belém</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Pescada</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>233.6</v>
+      </c>
+      <c r="D10" t="n">
+        <v>3098.5</v>
+      </c>
+      <c r="E10" t="n">
+        <v>187.7</v>
+      </c>
+      <c r="F10" t="n">
+        <v>2647.3</v>
+      </c>
+      <c r="G10" t="n">
+        <v>186.9</v>
+      </c>
+      <c r="H10" t="n">
+        <v>2178.5</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Augusto Corrêa</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Pargo</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>225.3</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2374.1</v>
+      </c>
+      <c r="E11" t="n">
+        <v>192</v>
+      </c>
+      <c r="F11" t="n">
+        <v>2760.6</v>
+      </c>
+      <c r="G11" t="n">
+        <v>167.5</v>
+      </c>
+      <c r="H11" t="n">
+        <v>2471.1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Augusto Corrêa</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Serra</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>117.7</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1113.8</v>
+      </c>
+      <c r="E12" t="n">
+        <v>145.3</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1884.6</v>
+      </c>
+      <c r="G12" t="n">
+        <v>134.8</v>
+      </c>
+      <c r="H12" t="n">
+        <v>1413.8</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Augusto Corrêa</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Pescada</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>163.3</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2515.1</v>
+      </c>
+      <c r="E13" t="n">
+        <v>168.1</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1824.6</v>
+      </c>
+      <c r="G13" t="n">
+        <v>152.1</v>
+      </c>
+      <c r="H13" t="n">
+        <v>1966.6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>codigo_coleta</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>estacao_periodo</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>comprimento_cm</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>peso_g</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>SERRA-2023-AUG</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>E04_Chuvosa</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>26.1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>213.2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>PESCADA-2021-AUG</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>E01_Seca</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>23.7</v>
+      </c>
+      <c r="E3" t="n">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>PESCADA-2023-AUG</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>E01_Chuvosa</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>32.1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>396.4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>PESCADA-2023-BEL</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>E01_Seca</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>43.2</v>
+      </c>
+      <c r="E5" t="n">
+        <v>818.1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>SERRA-2021-BEL</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>E03_Chuvosa</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>23.9</v>
+      </c>
+      <c r="E6" t="n">
+        <v>109.4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>PESCADA-2023-BEL</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>E02_Seca</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1163.1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>PESCADA-2021-VIG</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>E03_Seca</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>38</v>
+      </c>
+      <c r="E8" t="n">
+        <v>609.9</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>PESCADA-2023-BRA</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>E03_Chuvosa</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="E9" t="n">
+        <v>76.59999999999999</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>SERRA-2021-VIG</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>E02_Seca</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="E10" t="n">
+        <v>94.7</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>PARGO-2021-VIG</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>E06_Chuvosa</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>53</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1289.4</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>PESCADA-2021-AUG</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>E05_Seca</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="E12" t="n">
+        <v>839.9</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>PESCADA-2022-BEL</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>E05_Chuvosa</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="E13" t="n">
+        <v>101.4</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>SERRA-2023-BRA</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>E05_Seca</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>39.8</v>
+      </c>
+      <c r="E14" t="n">
+        <v>506.2</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>PESCADA-2021-BRA</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>E01_Seca</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>49.8</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1023.1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>PARGO-2023-BEL</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>E04_Seca</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>38</v>
+      </c>
+      <c r="E16" t="n">
+        <v>597.7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr codeName="Planilha3">

</xml_diff>